<commit_message>
Task 4 + 5 - sua lan 1
</commit_message>
<xml_diff>
--- a/CheckList.xlsx
+++ b/CheckList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rekkei_edu\FastAPI_CNTT6\ProjectFastAPI\event_management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F27BD56B-E742-45B2-B934-E8E408FCFD19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDD1B34-34B7-4CDD-B3DC-658B512286CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{D6DFB09B-CCBF-48AE-A752-2427DE08D5B3}"/>
   </bookViews>
@@ -77,9 +77,6 @@
     <t>Đăng ký tài khoản mới thành công</t>
   </si>
   <si>
-    <t>Body: Email chưa tồn tại, mật khẩu hợp lệ</t>
-  </si>
-  <si>
     <t>201 Created</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>Đăng ký trùng email đã có trong hệ thống</t>
   </si>
   <si>
-    <t>Body: Email đã tồn tại</t>
-  </si>
-  <si>
     <t>400 Bad Request</t>
   </si>
   <si>
@@ -101,9 +95,6 @@
     <t>Đăng nhập đúng thông tin</t>
   </si>
   <si>
-    <t>Body: Đúng email &amp; mật khẩu</t>
-  </si>
-  <si>
     <r>
       <t>200 OK</t>
     </r>
@@ -121,9 +112,6 @@
     <t>Đăng nhập sai mật khẩu</t>
   </si>
   <si>
-    <t>Body: Đúng email, sai mật khẩu</t>
-  </si>
-  <si>
     <t>401 Unauthorized</t>
   </si>
   <si>
@@ -137,6 +125,46 @@
   </si>
   <si>
     <r>
+      <t>201 Created</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (User là OWNER)</t>
+    </r>
+  </si>
+  <si>
+    <t>Tạo sự kiện không gửi Token</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Không gắn Header </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Authorization</t>
+    </r>
+  </si>
+  <si>
+    <t>401/403 Forbidden</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>Lấy danh sách sự kiện của tôi</t>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">Header: </t>
     </r>
     <r>
@@ -155,6 +183,351 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve"> User A</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>200 OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Chỉ sự kiện tham gia)</t>
+    </r>
+  </si>
+  <si>
+    <t>Tìm kiếm sự kiện theo tên</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Bearer Token</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">; Query: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>?name=Event</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>200 OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Lọc theo tên)</t>
+    </r>
+  </si>
+  <si>
+    <t>/events/{id}</t>
+  </si>
+  <si>
+    <t>Xem chi tiết sự kiện khi là Member/Owner</t>
+  </si>
+  <si>
+    <t>Header: Token User trong ban tổ chức</t>
+  </si>
+  <si>
+    <t>200 OK</t>
+  </si>
+  <si>
+    <t>Người ngoài sự kiện cố xem chi tiết</t>
+  </si>
+  <si>
+    <t>Header: Token User B (chưa tham gia Event)</t>
+  </si>
+  <si>
+    <t>403 Forbidden</t>
+  </si>
+  <si>
+    <t>PATCH</t>
+  </si>
+  <si>
+    <t>Owner cập nhật tên/mô tả sự kiện</t>
+  </si>
+  <si>
+    <t>Member cố tình sửa sự kiện</t>
+  </si>
+  <si>
+    <t>Header: Token của Member (không phải Owner)</t>
+  </si>
+  <si>
+    <t>Member</t>
+  </si>
+  <si>
+    <t>/events/{id}/members</t>
+  </si>
+  <si>
+    <t>Owner thêm user hợp lệ vào sự kiện</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token của Owner; Body: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>{"user_id": 2, "role": "MEMBER"}</t>
+    </r>
+  </si>
+  <si>
+    <t>Thêm trùng user đã có trong sự kiện</t>
+  </si>
+  <si>
+    <t>Header: Token của Owner; Body: User ID đã tồn tại</t>
+  </si>
+  <si>
+    <t>Thêm user không tồn tại trong hệ thống</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token của Owner; Body: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>{"user_id": 9999}</t>
+    </r>
+  </si>
+  <si>
+    <t>404 Not Found</t>
+  </si>
+  <si>
+    <t>Lấy danh sách thành viên trong sự kiện</t>
+  </si>
+  <si>
+    <t>Header: Token Member/Owner</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>/events/{id}/members/{u_id}</t>
+  </si>
+  <si>
+    <t>Owner xóa một Member ra khỏi sự kiện</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token Owner; Path: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>user_id</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> của Member</t>
+    </r>
+  </si>
+  <si>
+    <t>Cố xóa Owner duy nhất còn lại của Event</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token Owner; Path: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>user_id</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> của chính Owner</t>
+    </r>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>/events/{id}/event-tasks</t>
+  </si>
+  <si>
+    <t>Member tạo task và gán cho Member khác</t>
+  </si>
+  <si>
+    <t>Gán task cho user ngoài sự kiện</t>
+  </si>
+  <si>
+    <t>Lọc task theo status/priority và phân trang</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Query: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>?status=TODO&amp;page=1&amp;page_size=10</t>
+    </r>
+  </si>
+  <si>
+    <t>/event-tasks/{id}</t>
+  </si>
+  <si>
+    <t>Xem chi tiết công việc</t>
+  </si>
+  <si>
+    <t>Header: Token Member thuộc sự kiện</t>
+  </si>
+  <si>
+    <t>Assignee đổi trạng thái công việc (status)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token của Assignee; Body: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>{"status": "IN_PROGRESS"}</t>
+    </r>
+  </si>
+  <si>
+    <t>Assignee cố sửa trường cấm (ví dụ: title)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token Assignee; Body: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>{"title": "Đổi title"}</t>
+    </r>
+  </si>
+  <si>
+    <t>Member thường (không phải Owner) cố xóa task</t>
+  </si>
+  <si>
+    <t>Header: Token Member</t>
+  </si>
+  <si>
+    <t>Owner thực hiện xóa công việc</t>
+  </si>
+  <si>
+    <t>Header: Token Owner</t>
+  </si>
+  <si>
+    <t>Owner xóa toàn bộ sự kiện</t>
+  </si>
+  <si>
+    <t>Body: Email chưa tồn tại, mật khẩu hợp lệ {
+  "email": "owner@gmail.com",
+  "password": "Password123@",
+  "full_name": "Nguyễn Văn Chủ"
+}</t>
+  </si>
+  <si>
+    <t>Body: Email đã tồn tại {
+  "email": "owner@gmail.com",
+  "password": "Password123@",
+  "full_name": "Nguyễn Văn Trùng"
+}</t>
+  </si>
+  <si>
+    <t>Body: Đúng email &amp; mật khẩu {
+  "email": "owner@gmail.com",
+  "password": "Password123@"
+}</t>
+  </si>
+  <si>
+    <t>Body: Đúng email, sai mật khẩu {
+  "email": "owner@gmail.com",
+  "password": "SaiPassword123"
+}</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>Bearer Token</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve"> User A; Body: </t>
     </r>
     <r>
@@ -164,12 +537,10 @@
         <rFont val="Google Sans Text"/>
         <family val="2"/>
       </rPr>
-      <t>{"name": "Event A"}</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>201 Created</t>
+      <t>{
+  "name": "Tech Expo 2026",
+  "description": "Hội thảo công nghệ AI"
+}</t>
     </r>
     <r>
       <rPr>
@@ -178,15 +549,12 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> (User là OWNER)</t>
-    </r>
-  </si>
-  <si>
-    <t>Tạo sự kiện không gửi Token</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Không gắn Header </t>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token của Owner; Body: </t>
     </r>
     <r>
       <rPr>
@@ -195,21 +563,14 @@
         <rFont val="Google Sans Text"/>
         <family val="2"/>
       </rPr>
-      <t>Authorization</t>
-    </r>
-  </si>
-  <si>
-    <t>401/403 Forbidden</t>
-  </si>
-  <si>
-    <t>GET</t>
-  </si>
-  <si>
-    <t>Lấy danh sách sự kiện của tôi</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: </t>
+      <t>{
+  "name": "Tech Expo 2026 Cập Nhật"
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token Member; Body: </t>
     </r>
     <r>
       <rPr>
@@ -218,7 +579,7 @@
         <rFont val="Google Sans Text"/>
         <family val="2"/>
       </rPr>
-      <t>Bearer Token</t>
+      <t>assignee_id</t>
     </r>
     <r>
       <rPr>
@@ -227,29 +588,18 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> User A</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>200 OK</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Chỉ sự kiện tham gia)</t>
-    </r>
-  </si>
-  <si>
-    <t>Tìm kiếm sự kiện theo tên</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: </t>
+      <t xml:space="preserve"> thuộc Event {
+  "title": "Thiết kế Poster",
+  "description": "Làm poster chính kích thước A1",
+  "priority": "HIGH",
+  "due_date": "2026-09-10T18:00:00",
+  "assignee_id": 2
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Header: Token Member; Body: </t>
     </r>
     <r>
       <rPr>
@@ -258,333 +608,11 @@
         <rFont val="Google Sans Text"/>
         <family val="2"/>
       </rPr>
-      <t>Bearer Token</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">; Query: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>?name=Event</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>200 OK</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Lọc theo tên)</t>
-    </r>
-  </si>
-  <si>
-    <t>/events/{id}</t>
-  </si>
-  <si>
-    <t>Xem chi tiết sự kiện khi là Member/Owner</t>
-  </si>
-  <si>
-    <t>Header: Token User trong ban tổ chức</t>
-  </si>
-  <si>
-    <t>200 OK</t>
-  </si>
-  <si>
-    <t>Người ngoài sự kiện cố xem chi tiết</t>
-  </si>
-  <si>
-    <t>Header: Token User B (chưa tham gia Event)</t>
-  </si>
-  <si>
-    <t>403 Forbidden</t>
-  </si>
-  <si>
-    <t>PATCH</t>
-  </si>
-  <si>
-    <t>Owner cập nhật tên/mô tả sự kiện</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token của Owner; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>{"name": "New Name"}</t>
-    </r>
-  </si>
-  <si>
-    <t>Member cố tình sửa sự kiện</t>
-  </si>
-  <si>
-    <t>Header: Token của Member (không phải Owner)</t>
-  </si>
-  <si>
-    <t>Member</t>
-  </si>
-  <si>
-    <t>/events/{id}/members</t>
-  </si>
-  <si>
-    <t>Owner thêm user hợp lệ vào sự kiện</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token của Owner; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>{"user_id": 2, "role": "MEMBER"}</t>
-    </r>
-  </si>
-  <si>
-    <t>Thêm trùng user đã có trong sự kiện</t>
-  </si>
-  <si>
-    <t>Header: Token của Owner; Body: User ID đã tồn tại</t>
-  </si>
-  <si>
-    <t>Thêm user không tồn tại trong hệ thống</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token của Owner; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>{"user_id": 9999}</t>
-    </r>
-  </si>
-  <si>
-    <t>404 Not Found</t>
-  </si>
-  <si>
-    <t>Lấy danh sách thành viên trong sự kiện</t>
-  </si>
-  <si>
-    <t>Header: Token Member/Owner</t>
-  </si>
-  <si>
-    <t>DELETE</t>
-  </si>
-  <si>
-    <t>/events/{id}/members/{u_id}</t>
-  </si>
-  <si>
-    <t>Owner xóa một Member ra khỏi sự kiện</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token Owner; Path: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>user_id</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> của Member</t>
-    </r>
-  </si>
-  <si>
-    <t>Cố xóa Owner duy nhất còn lại của Event</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token Owner; Path: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>user_id</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> của chính Owner</t>
-    </r>
-  </si>
-  <si>
-    <t>Task</t>
-  </si>
-  <si>
-    <t>/events/{id}/event-tasks</t>
-  </si>
-  <si>
-    <t>Member tạo task và gán cho Member khác</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token Member; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>assignee_id</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> thuộc Event</t>
-    </r>
-  </si>
-  <si>
-    <t>Gán task cho user ngoài sự kiện</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token Member; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>assignee_id</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> không trong Event</t>
-    </r>
-  </si>
-  <si>
-    <t>Lọc task theo status/priority và phân trang</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Query: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>?status=TODO&amp;page=1&amp;page_size=10</t>
-    </r>
-  </si>
-  <si>
-    <t>/event-tasks/{id}</t>
-  </si>
-  <si>
-    <t>Xem chi tiết công việc</t>
-  </si>
-  <si>
-    <t>Header: Token Member thuộc sự kiện</t>
-  </si>
-  <si>
-    <t>Assignee đổi trạng thái công việc (status)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token của Assignee; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>{"status": "IN_PROGRESS"}</t>
-    </r>
-  </si>
-  <si>
-    <t>Assignee cố sửa trường cấm (ví dụ: title)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Header: Token Assignee; Body: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>{"title": "Đổi title"}</t>
-    </r>
-  </si>
-  <si>
-    <t>Member thường (không phải Owner) cố xóa task</t>
-  </si>
-  <si>
-    <t>Header: Token Member</t>
-  </si>
-  <si>
-    <t>Owner thực hiện xóa công việc</t>
-  </si>
-  <si>
-    <t>Header: Token Owner</t>
-  </si>
-  <si>
-    <t>Owner xóa toàn bộ sự kiện</t>
+      <t>{
+  "title": "Task Lỗi",
+  "assignee_id": 3
+}</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1044,7 +1072,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.5" thickBot="1">
+    <row r="2" spans="1:8" ht="186" thickBot="1">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1061,16 +1089,16 @@
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="43.5" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="171.75" thickBot="1">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1084,19 +1112,19 @@
         <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="H3" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="29.25" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="143.25" thickBot="1">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1107,22 +1135,22 @@
         <v>9</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="43.5" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="143.25" thickBot="1">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1133,45 +1161,45 @@
         <v>9</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="57.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="129" thickBot="1">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="43.5" thickBot="1">
@@ -1179,25 +1207,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="43.5" thickBot="1">
@@ -1205,25 +1233,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="43.5" thickBot="1">
@@ -1231,25 +1259,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.5" thickBot="1">
@@ -1257,25 +1285,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="43.5" thickBot="1">
@@ -1283,51 +1311,51 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="G11" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="57.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="100.5" thickBot="1">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="57.75" thickBot="1">
@@ -1335,25 +1363,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="72" thickBot="1">
@@ -1361,25 +1389,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="57.75" thickBot="1">
@@ -1387,25 +1415,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="57.75" thickBot="1">
@@ -1413,25 +1441,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="G16" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="43.5" thickBot="1">
@@ -1439,25 +1467,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="57.75" thickBot="1">
@@ -1465,25 +1493,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="57.75" thickBot="1">
@@ -1491,77 +1519,77 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="57.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="243" thickBot="1">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="72" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="86.25" thickBot="1">
       <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="57.75" thickBot="1">
@@ -1569,25 +1597,25 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="43.5" thickBot="1">
@@ -1595,25 +1623,25 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="E23" s="2" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="72" thickBot="1">
@@ -1621,25 +1649,25 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="57.75" thickBot="1">
@@ -1647,25 +1675,25 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="E25" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="57.75" thickBot="1">
@@ -1673,25 +1701,25 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="G26" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="43.5" thickBot="1">
@@ -1699,25 +1727,25 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="E27" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="29.25" thickBot="1">
@@ -1725,25 +1753,25 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>